<commit_message>
Afegits destacades, notes i altres
</commit_message>
<xml_diff>
--- a/Programa/seguiment_preus.xlsx
+++ b/Programa/seguiment_preus.xlsx
@@ -11,7 +11,11 @@
     <sheet name="Integral 0.75cl" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Rosé 0.75cl" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Brut Nature 0.75cl'!$A$2:$H$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Integral 0.75cl'!$A$2:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Rosé 0.75cl'!$A$2:$H$4</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -21,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="+0.0%;-0.0%"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,23 +35,53 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <b val="1"/>
     </font>
     <font>
-      <color rgb="00007A33"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <i val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00007A33"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+        <bgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CCFF66"/>
+        <bgColor rgb="00CCFF66"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F4FF"/>
+        <bgColor rgb="00F0F4FF"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -68,13 +102,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="4" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -440,13 +488,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D40"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,630 +512,1013 @@
           <t>% vs preu botiga</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Preu</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Preu</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Preu</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Winepalace</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>-0.002958579881656637</v>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="6" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="6" t="n">
+        <v>16.85</v>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Vivónium</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B4" s="9" t="n">
         <v>-0.229585798816568</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C4" s="6" t="n">
         <v>13.02</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="6" t="n">
         <v>13.02</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="6" t="n">
+        <v>13.02</v>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Cash Montseny</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B5" s="9" t="n">
         <v>-0.1686390532544378</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C5" s="6" t="n">
         <v>14.05</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="6" t="n">
         <v>14.05</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="6" t="n">
+        <v>14.05</v>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Bodega Vidal</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B6" s="9" t="n">
         <v>-0.1579881656804733</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C6" s="6" t="n">
         <v>14.23</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D6" s="7" t="n"/>
+      <c r="E6" s="6" t="n">
         <v>14.23</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="6" t="n">
+        <v>14.23</v>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>EnterWine</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B7" s="9" t="n">
         <v>-0.1007336686390531</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C7" s="6" t="n">
         <v>15.197601</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="6" t="n">
         <v>15.197601</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="6" t="n">
+        <v>15.197601</v>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Cal Angel</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B8" s="9" t="n">
         <v>-0.09822485207100583</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C8" s="6" t="n">
         <v>15.24</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D8" s="7" t="n"/>
+      <c r="E8" s="6" t="n">
         <v>15.24</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="F8" s="7" t="n"/>
+      <c r="G8" s="6" t="n">
+        <v>15.24</v>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Sorli</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B9" s="9" t="n">
         <v>-0.09526627218934909</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C9" s="10" t="n">
         <v>15.29</v>
       </c>
-      <c r="D7" s="4" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
+      <c r="D9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Carviresa</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>-0.08402366863905315</v>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>15.48</v>
+      </c>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="6" t="n">
+        <v>15.48</v>
+      </c>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="6" t="n">
+        <v>15.48</v>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>EnBotella</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B11" s="9" t="n">
         <v>-0.08402366863905315</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C11" s="6" t="n">
         <v>15.48</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D11" s="7" t="n"/>
+      <c r="E11" s="6" t="n">
         <v>15.48</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Carviresa</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>-0.08402366863905315</v>
-      </c>
-      <c r="C9" s="3" t="n">
+      <c r="F11" s="7" t="n"/>
+      <c r="G11" s="6" t="n">
         <v>15.48</v>
       </c>
-      <c r="D9" s="3" t="n">
-        <v>15.48</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Degusta'm</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>-0.08284023668639046</v>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="D12" s="7" t="n"/>
+      <c r="E12" s="6" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="F12" s="7" t="n"/>
+      <c r="G12" s="6" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>La Vinateria</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B13" s="9" t="n">
         <v>-0.08284023668639046</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C13" s="6" t="n">
         <v>15.5</v>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D13" s="7" t="n"/>
+      <c r="E13" s="6" t="n">
         <v>15.5</v>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>Degusta'm</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>-0.08284023668639046</v>
-      </c>
-      <c r="C11" s="3" t="n">
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="6" t="n">
         <v>15.5</v>
       </c>
-      <c r="D11" s="3" t="n">
-        <v>15.5</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Vins a casa</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B14" s="9" t="n">
         <v>-0.07396449704142002</v>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C14" s="6" t="n">
         <v>16.3</v>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="6" t="n">
         <v>15.65</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="6" t="n">
+        <v>15.65</v>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Grau Online</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B15" s="9" t="n">
         <v>-0.07218934911242597</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C15" s="6" t="n">
         <v>15.68</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D15" s="7" t="n"/>
+      <c r="E15" s="6" t="n">
         <v>15.68</v>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="F15" s="7" t="n"/>
+      <c r="G15" s="6" t="n">
+        <v>15.68</v>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
         <is>
           <t>Bonpreu Esclat</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B16" s="9" t="n">
         <v>-0.07159763313609463</v>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C16" s="6" t="n">
         <v>15.69</v>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="6" t="n">
         <v>15.69</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="6" t="n">
+        <v>15.69</v>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Decantalo</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>-0.06804733727810643</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="D17" s="7" t="n"/>
+      <c r="F17" s="7" t="n"/>
+      <c r="H17" s="7" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Vinissimus</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>-0.06804733727810643</v>
+      </c>
+      <c r="C18" s="6" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="D18" s="7" t="n"/>
+      <c r="E18" s="6" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="F18" s="7" t="n"/>
+      <c r="G18" s="6" t="n">
+        <v>15.75</v>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Vinos en Casa</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B19" s="9" t="n">
         <v>-0.06804733727810643</v>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C19" s="6" t="n">
         <v>16.3</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D19" s="7" t="n"/>
+      <c r="E19" s="6" t="n">
         <v>15.75</v>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>Vinissimus</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>-0.06804733727810643</v>
-      </c>
-      <c r="C16" s="3" t="n">
+      <c r="F19" s="7" t="n"/>
+      <c r="G19" s="6" t="n">
         <v>15.75</v>
       </c>
-      <c r="D16" s="3" t="n">
-        <v>15.75</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>Decantalo</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>-0.06804733727810643</v>
-      </c>
-      <c r="C17" s="4" t="n">
-        <v>15.75</v>
-      </c>
-      <c r="D17" s="4" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>TotVi</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B20" s="9" t="n">
         <v>-0.06508875739644958</v>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C20" s="6" t="n">
         <v>15.8</v>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D20" s="7" t="n"/>
+      <c r="E20" s="6" t="n">
         <v>15.8</v>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+      <c r="F20" s="7" t="n"/>
+      <c r="G20" s="6" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="H20" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Verema i Collita</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>-0.05917159763313599</v>
+      </c>
+      <c r="C21" s="6" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="D21" s="7" t="n"/>
+      <c r="E21" s="6" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="F21" s="7" t="n"/>
+      <c r="G21" s="6" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Vinos Barcelona</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B22" s="9" t="n">
         <v>-0.05917159763313599</v>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C22" s="6" t="n">
         <v>15.9</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="6" t="n">
         <v>15.9</v>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr">
-        <is>
-          <t>Verema i Collita</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>-0.05917159763313599</v>
-      </c>
-      <c r="C20" s="3" t="n">
+      <c r="F22" s="7" t="n"/>
+      <c r="G22" s="6" t="n">
         <v>15.9</v>
       </c>
-      <c r="D20" s="3" t="n">
-        <v>15.9</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Vinos  Online</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B23" s="9" t="n">
         <v>-0.04674556213017747</v>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C23" s="10" t="n">
         <v>16.11</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D23" s="7" t="n"/>
+      <c r="E23" s="6" t="n">
         <v>16.11</v>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
+      <c r="F23" s="7" t="n"/>
+      <c r="G23" s="6" t="n">
+        <v>16.11</v>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>Vino Premier</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B24" s="9" t="n">
         <v>-0.03846153846153838</v>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C24" s="6" t="n">
         <v>16.25</v>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D24" s="7" t="n"/>
+      <c r="E24" s="6" t="n">
         <v>16.25</v>
       </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="6" t="n">
+        <v>16.25</v>
+      </c>
+      <c r="H24" s="7" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Vinomada</t>
         </is>
       </c>
-      <c r="B23" s="2" t="n">
+      <c r="B25" s="9" t="n">
         <v>-0.03846153846153838</v>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C25" s="6" t="n">
         <v>16.25</v>
       </c>
-      <c r="D23" s="4" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+      <c r="D25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="H25" s="7" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>VinoVí</t>
         </is>
       </c>
-      <c r="B24" s="2" t="n">
+      <c r="B26" s="9" t="n">
         <v>-0.03550295857988153</v>
       </c>
-      <c r="C24" s="3" t="n">
+      <c r="C26" s="6" t="n">
         <v>16.3</v>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D26" s="7" t="n"/>
+      <c r="E26" s="6" t="n">
         <v>16.3</v>
       </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+      <c r="F26" s="7" t="n"/>
+      <c r="G26" s="6" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Vins Noe</t>
         </is>
       </c>
-      <c r="B25" s="2" t="n">
+      <c r="B27" s="9" t="n">
         <v>-0.03550295857988153</v>
       </c>
-      <c r="C25" s="4" t="n">
+      <c r="C27" s="10" t="n">
         <v>16.3</v>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D27" s="7" t="n"/>
+      <c r="E27" s="6" t="n">
         <v>16.3</v>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+      <c r="F27" s="7" t="n"/>
+      <c r="G27" s="6" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>Bodeboca</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
+      <c r="B28" s="9" t="n">
         <v>-0.02958579881656805</v>
       </c>
-      <c r="C26" s="4" t="n">
+      <c r="C28" s="10" t="n">
         <v>16.4</v>
       </c>
-      <c r="D26" s="4" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+      <c r="D28" s="7" t="n"/>
+      <c r="F28" s="7" t="n"/>
+      <c r="H28" s="7" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>La Branca</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n">
+      <c r="B29" s="9" t="n">
         <v>-0.02958579881656805</v>
       </c>
-      <c r="C27" s="3" t="n">
+      <c r="C29" s="6" t="n">
         <v>16.4</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D29" s="7" t="n"/>
+      <c r="E29" s="6" t="n">
         <v>16.4</v>
       </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+      <c r="F29" s="7" t="n"/>
+      <c r="G29" s="6" t="n">
+        <v>16.4</v>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>TendaVins</t>
         </is>
       </c>
-      <c r="B28" s="2" t="n">
+      <c r="B30" s="9" t="n">
         <v>-0.02366863905325435</v>
       </c>
-      <c r="C28" s="3" t="n">
+      <c r="C30" s="6" t="n">
         <v>16.5</v>
       </c>
-      <c r="D28" s="3" t="n">
+      <c r="D30" s="7" t="n"/>
+      <c r="E30" s="6" t="n">
         <v>16.5</v>
       </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+      <c r="F30" s="7" t="n"/>
+      <c r="G30" s="6" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="H30" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>Cal Feru</t>
         </is>
       </c>
-      <c r="B29" s="2" t="n">
+      <c r="B31" s="9" t="n">
         <v>-0.01479289940828402</v>
       </c>
-      <c r="C29" s="3" t="n">
+      <c r="C31" s="6" t="n">
         <v>16.65</v>
       </c>
-      <c r="D29" s="3" t="n">
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="6" t="n">
         <v>16.65</v>
       </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="6" t="n">
+        <v>16.65</v>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Santa Cecilia</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="n">
+        <v>-0.008875739644970331</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>16.75</v>
+      </c>
+      <c r="D32" s="7" t="n"/>
+      <c r="E32" s="6" t="n">
+        <v>16.75</v>
+      </c>
+      <c r="F32" s="7" t="n"/>
+      <c r="G32" s="6" t="n">
+        <v>16.75</v>
+      </c>
+      <c r="H32" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>Vinos Baco</t>
         </is>
       </c>
-      <c r="B30" s="2" t="n">
+      <c r="B33" s="9" t="n">
         <v>-0.008875739644970331</v>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C33" s="6" t="n">
         <v>16.75</v>
       </c>
-      <c r="D30" s="3" t="n">
+      <c r="D33" s="7" t="n"/>
+      <c r="E33" s="6" t="n">
         <v>16.75</v>
       </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>Santa Cecilia</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>-0.008875739644970331</v>
-      </c>
-      <c r="C31" s="3" t="n">
+      <c r="F33" s="7" t="n"/>
+      <c r="G33" s="6" t="n">
         <v>16.75</v>
       </c>
-      <c r="D31" s="3" t="n">
-        <v>16.75</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>Winepalace</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n">
-        <v>-0.002958579881656637</v>
-      </c>
-      <c r="C32" s="3" t="n">
-        <v>16.85</v>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>16.85</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="1" t="inlineStr">
+      <c r="H33" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="8" t="inlineStr">
         <is>
           <t>Ametller Origen</t>
         </is>
       </c>
-      <c r="B33" s="5" t="n">
+      <c r="B34" s="11" t="n">
         <v>0.002958579881656847</v>
       </c>
-      <c r="C33" s="4" t="n">
+      <c r="C34" s="10" t="n">
         <v>16.95</v>
       </c>
-      <c r="D33" s="4" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+      <c r="D34" s="7" t="n"/>
+      <c r="F34" s="7" t="n"/>
+      <c r="H34" s="7" t="n"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>Caprabo</t>
         </is>
       </c>
-      <c r="B34" s="5" t="n">
+      <c r="B35" s="11" t="n">
         <v>0.002958579881656847</v>
       </c>
-      <c r="C34" s="3" t="n">
+      <c r="C35" s="6" t="n">
         <v>16.95</v>
       </c>
-      <c r="D34" s="3" t="n">
+      <c r="D35" s="7" t="n"/>
+      <c r="E35" s="6" t="n">
         <v>16.95</v>
       </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="1" t="inlineStr">
+      <c r="F35" s="7" t="n"/>
+      <c r="G35" s="6" t="n">
+        <v>16.95</v>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>Celler de gelida</t>
         </is>
       </c>
-      <c r="B35" s="5" t="n">
+      <c r="B36" s="11" t="n">
         <v>0.002958579881656847</v>
       </c>
-      <c r="C35" s="3" t="n">
+      <c r="C36" s="6" t="n">
         <v>16.95</v>
       </c>
-      <c r="D35" s="3" t="n">
+      <c r="D36" s="7" t="n"/>
+      <c r="E36" s="6" t="n">
         <v>16.95</v>
       </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="1" t="inlineStr">
+      <c r="F36" s="7" t="n"/>
+      <c r="G36" s="6" t="n">
+        <v>16.95</v>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>Condis</t>
         </is>
       </c>
-      <c r="B36" s="5" t="n">
+      <c r="B37" s="11" t="n">
         <v>0.002958579881656847</v>
       </c>
-      <c r="C36" s="4" t="n">
+      <c r="C37" s="10" t="n">
         <v>16.95</v>
       </c>
-      <c r="D36" s="4" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="inlineStr">
+      <c r="D37" s="7" t="n"/>
+      <c r="F37" s="7" t="n"/>
+      <c r="H37" s="7" t="n"/>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>La Fuente</t>
         </is>
       </c>
-      <c r="B37" s="5" t="n">
+      <c r="B38" s="11" t="n">
         <v>0.0325443786982249</v>
       </c>
-      <c r="C37" s="3" t="n">
+      <c r="C38" s="6" t="n">
         <v>17.45</v>
       </c>
-      <c r="D37" s="3" t="n">
+      <c r="D38" s="7" t="n"/>
+      <c r="E38" s="6" t="n">
         <v>17.45</v>
       </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="inlineStr">
+      <c r="F38" s="7" t="n"/>
+      <c r="G38" s="6" t="n">
+        <v>17.45</v>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>Descorcha y bebe</t>
         </is>
       </c>
-      <c r="B38" s="5" t="n">
+      <c r="B39" s="11" t="n">
         <v>0.06213017751479295</v>
       </c>
-      <c r="C38" s="3" t="n">
+      <c r="C39" s="6" t="n">
         <v>17.95</v>
       </c>
-      <c r="D38" s="3" t="n">
+      <c r="D39" s="7" t="n"/>
+      <c r="E39" s="6" t="n">
         <v>17.95</v>
       </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="1" t="inlineStr">
+      <c r="F39" s="7" t="n"/>
+      <c r="G39" s="6" t="n">
+        <v>17.95</v>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>Móntatelo en casa</t>
         </is>
       </c>
-      <c r="B39" s="5" t="n">
+      <c r="B40" s="11" t="n">
         <v>0.1189349112426036</v>
       </c>
-      <c r="C39" s="3" t="n">
+      <c r="C40" s="6" t="n">
         <v>18.91</v>
       </c>
-      <c r="D39" s="3" t="n">
+      <c r="D40" s="7" t="n"/>
+      <c r="E40" s="6" t="n">
         <v>18.91</v>
       </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="inlineStr">
+      <c r="F40" s="7" t="n"/>
+      <c r="G40" s="6" t="n">
+        <v>18.91</v>
+      </c>
+      <c r="H40" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="8" t="inlineStr">
         <is>
           <t>Private Celler</t>
         </is>
       </c>
-      <c r="B40" s="5" t="n">
+      <c r="B41" s="11" t="n">
         <v>0.121301775147929</v>
       </c>
-      <c r="C40" s="3" t="n">
+      <c r="C41" s="6" t="n">
         <v>18.95</v>
       </c>
-      <c r="D40" s="3" t="n">
+      <c r="D41" s="7" t="n"/>
+      <c r="E41" s="6" t="n">
         <v>18.95</v>
       </c>
+      <c r="F41" s="7" t="n"/>
+      <c r="G41" s="6" t="n">
+        <v>18.95</v>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:H41"/>
+  <mergeCells count="5">
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1094,12 +1529,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1113,39 +1551,91 @@
           <t>% vs preu botiga</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Preu</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Preu</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>Bonpreu Esclat</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B3" s="9" t="n">
         <v>-0.1021390374331551</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C3" s="6" t="n">
         <v>16.79</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="6" t="n">
+        <v>16.79</v>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Cal Feru</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B4" s="9" t="n">
         <v>-0.02139037433155073</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C4" s="6" t="n">
         <v>18.3</v>
       </c>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="6" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:F4"/>
+  <mergeCells count="4">
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1156,13 +1646,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1176,48 +1670,112 @@
           <t>% vs preu botiga</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Preu</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Preu</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Preu</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Bonpreu Esclat</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>-0.05614973262032089</v>
+      </c>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="6" t="n">
+        <v>17.65</v>
+      </c>
+      <c r="F3" s="7" t="n"/>
+      <c r="G3" s="6" t="n">
+        <v>17.65</v>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Vinissimus</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
-        <v>-0.1021390374331551</v>
-      </c>
-      <c r="C2" s="3" t="n">
+      <c r="B4" s="11" t="n">
+        <v>0.02406417112299462</v>
+      </c>
+      <c r="C4" s="6" t="n">
         <v>17.65</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="6" t="n">
         <v>16.79</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Bonpreu Esclat</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>-0.05614973262032089</v>
-      </c>
-      <c r="C3" s="4" t="inlineStr"/>
-      <c r="D3" s="3" t="n">
-        <v>17.65</v>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="6" t="n">
+        <v>19.15</v>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Campanya estiu</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:H4"/>
+  <mergeCells count="5">
+    <mergeCell ref="C1:D1"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="A1:A2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>